<commit_message>
feat(task2,task3): 完整版 — 多轮对话修复 / rank 回退 / RAG 去噪 / 附件7 JSON / 图片嵌入
任务二升级：
- 新增 field_schema.py 统一字段元数据 (table/column/unit/kind)，60+ 同义词
- dialogue.py：上一轮澄清 → 本轮补信息可沿用前一 intent 类型
- answer_q4：rank 无公司时也能出 SQL（默认 FY + LIMIT 10）；rule_answer 按 kind 格式化，带单位与百分比
- chart.py：percent y 轴 formatter + bar 柱顶标注 + 多 series 分组修复
- prompts.py：追加 4 条 NL→SQL few-shot
- 回答 JSON 严格按附件 7 表 2：{问题编号, 问题类型, 子问题[{Q,A,SQL,image}]}

任务三升级：
- rag_index：跳过封面页 + 免责声明过滤；chunk 300/60；min_score 阈值 + stock boost
- paper_image.py 新增：PyMuPDF 渲染 PDF 页到 result/refs/*.jpg
- attribution：关键词提取 + LLM query 改写 + (paper,page) 去重 + LLM 归因总结
- planner：多意图规则 (rank+compare / trend+attribution); 结构化空时自动追加 attribution
- answer_q6：y_field 在加 _period 前固化；回答 JSON 对齐附件 7 表 5；references 含 paper_image

Excel 输出：
- excel_io.write_task_results_with_images 支持 inline 图表 + 研报截图两列
- result_2.xlsx：7 列（含"图表"），每题嵌入子问题最末图
- result_3.xlsx：8 列（含"图表"、"研报截图"），首张 paper_image 嵌入

https://claude.ai/code/session_0144kjAFsCgPBbgaUDoRdnkk
</commit_message>
<xml_diff>
--- a/result/result_2.xlsx
+++ b/result/result_2.xlsx
@@ -127,6 +127,61 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2286000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2286000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -416,15 +471,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
     <col width="80" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -458,8 +514,13 @@
           <t>回答</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>图表</t>
+        </is>
+      </c>
     </row>
-    <row r="2">
+    <row r="2" ht="120" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>B1001</t>
@@ -493,13 +554,13 @@
   "子问题": [
     {
       "Q": "金花股份利润总额是多少",
-      "A": "共 12 行：('金花股份', 2022, 'FY', None); ('金花股份', 2023, 'Q1', None); ('金花股份', 2023, 'HY', None)",
+      "A": "金花股份的利润总额从2024三季报的 3,245.72 万元 变化到2025三季报的 3,533.59 万元（+8.87%）",
       "SQL": "SELECT stock_abbr, report_year, report_period, total_profit FROM income_sheet WHERE (stock_abbr='金花股份') ORDER BY stock_code, report_year, CASE report_period WHEN 'Q1' THEN 1 WHEN 'HY' THEN 2 WHEN 'Q3' THEN 3 WHEN 'FY' THEN 4 END",
       "image": "B1001_1.jpg"
     },
     {
       "Q": "2025年第三季度的",
-      "A": "共 1 行：('金花股份', 2025, 'Q3', 3533.59)",
+      "A": "金花股份 2025三季报的利润总额为 3,533.59 万元",
       "SQL": "SELECT stock_abbr, report_year, report_period, total_profit FROM income_sheet WHERE (stock_abbr='金花股份') AND report_year IN (2025) AND report_period IN ('Q3') ORDER BY stock_code, report_year, CASE report_period WHEN 'Q1' THEN 1 WHEN 'HY' THEN 2 WHEN 'Q3' THEN 3 WHEN 'FY' THEN 4 END",
       "image": "B1001_2.jpg"
     }
@@ -507,8 +568,13 @@
 }</t>
         </is>
       </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>B1001_2.jpg</t>
+        </is>
+      </c>
     </row>
-    <row r="3">
+    <row r="3" ht="120" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>B1002</t>
@@ -542,7 +608,7 @@
   "子问题": [
     {
       "Q": "金花股份近几年的利润总额变化趋势是什么样的",
-      "A": "共 12 行：('金花股份', 2022, 'FY', None); ('金花股份', 2023, 'Q1', None); ('金花股份', 2023, 'HY', None)",
+      "A": "金花股份的利润总额从2024三季报的 3,245.72 万元 变化到2025三季报的 3,533.59 万元（+8.87%）",
       "SQL": "SELECT stock_abbr, report_year, report_period, total_profit FROM income_sheet WHERE (stock_abbr='金花股份') ORDER BY stock_code, report_year, CASE report_period WHEN 'Q1' THEN 1 WHEN 'HY' THEN 2 WHEN 'Q3' THEN 3 WHEN 'FY' THEN 4 END",
       "image": "B1002_1.jpg"
     }
@@ -550,8 +616,14 @@
 }</t>
         </is>
       </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>B1002_1.jpg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>